<commit_message>
added scenario 2 as it is needed for baseline
</commit_message>
<xml_diff>
--- a/notebooks/CalSim3GroundWaterDataExtractionInitFile_v1.xlsx
+++ b/notebooks/CalSim3GroundWaterDataExtractionInitFile_v1.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F1C3EF1-90F3-4CBC-8F34-F22BAAB91097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96085474-AFFF-4CE1-96C6-9795E96A376A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -231,25 +231,25 @@
     <t>E266</t>
   </si>
   <si>
-    <t>A25</t>
-  </si>
-  <si>
-    <t>B25</t>
-  </si>
-  <si>
-    <t>C25</t>
-  </si>
-  <si>
-    <t>G25</t>
-  </si>
-  <si>
-    <t>H25</t>
-  </si>
-  <si>
-    <t>I25</t>
-  </si>
-  <si>
-    <t>J25</t>
+    <t>A26</t>
+  </si>
+  <si>
+    <t>B26</t>
+  </si>
+  <si>
+    <t>C26</t>
+  </si>
+  <si>
+    <t>G26</t>
+  </si>
+  <si>
+    <t>H26</t>
+  </si>
+  <si>
+    <t>I26</t>
+  </si>
+  <si>
+    <t>J26</t>
   </si>
 </sst>
 </file>

</xml_diff>